<commit_message>
AFLP Moto Manager : corrections de recette, documentation, résultats
- dotation en écart : part reçue comptée dans l'avance à apurer (SQL, cœur, tests)
- en-tête mobile 390 px, libellés de la file de synchronisation
- guides, rapport de sécurité, rapport d'exécution, matrice de substitution
- résultats : serveur 186/186, navigateur 54/54, unitaires 10/10, 0 nouveau défaut

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01YFAq1f7wanW5Hm7vGnu6CV
</commit_message>
<xml_diff>
--- a/tests/moto/resultats/export-pilotage-e2e.xlsx
+++ b/tests/moto/resultats/export-pilotage-e2e.xlsx
@@ -479,7 +479,7 @@
         <v>UH SAKASSOU E2E FICTIF</v>
       </c>
       <c r="K2" t="str">
-        <v>2026-10-30T23:31:47.677454+00:00</v>
+        <v>2026-10-30T23:38:56.983553+00:00</v>
       </c>
       <c r="L2">
         <v>160</v>
@@ -530,7 +530,7 @@
         <v>Immobilisée</v>
       </c>
       <c r="E2" t="str">
-        <v>2026-10-30T23:31:55.082515+00:00</v>
+        <v>2026-10-30T23:39:04.193383+00:00</v>
       </c>
       <c r="F2" t="str">
         <v/>
@@ -563,7 +563,7 @@
         <v>Observation limitée : 1 moto(s), 1 intervalle(s) plein à plein. Ces valeurs décrivent le pilote ; elles ne constituent pas une référence statistique.</v>
       </c>
       <c r="B2" t="str">
-        <v>2026-10-30T23:32:06.417Z</v>
+        <v>2026-10-30T23:39:14.990Z</v>
       </c>
       <c r="C2" t="str">
         <v>BM E2E FICTIF</v>
@@ -617,7 +617,7 @@
         <v>3.5</v>
       </c>
       <c r="F2" t="str">
-        <v>2026-10-30T23:31:53.645+00:00</v>
+        <v>2026-10-30T23:39:02.928+00:00</v>
       </c>
     </row>
   </sheetData>
@@ -851,7 +851,7 @@
         <v>0</v>
       </c>
       <c r="F2">
-        <v>0</v>
+        <v>9900</v>
       </c>
       <c r="G2">
         <v>100</v>
@@ -866,7 +866,7 @@
         <v>0</v>
       </c>
       <c r="K2">
-        <v>-2550</v>
+        <v>7350</v>
       </c>
       <c r="L2">
         <v>0</v>

</xml_diff>

<commit_message>
AFLP Moto Manager : contrôle de départ bloqué sur moto immobilisée côté serveur, captures rafraîchies
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01YFAq1f7wanW5Hm7vGnu6CV
</commit_message>
<xml_diff>
--- a/tests/moto/resultats/export-pilotage-e2e.xlsx
+++ b/tests/moto/resultats/export-pilotage-e2e.xlsx
@@ -479,7 +479,7 @@
         <v>UH SAKASSOU E2E FICTIF</v>
       </c>
       <c r="K2" t="str">
-        <v>2026-10-30T23:38:56.983553+00:00</v>
+        <v>2026-10-30T23:47:33.091473+00:00</v>
       </c>
       <c r="L2">
         <v>160</v>
@@ -530,7 +530,7 @@
         <v>Immobilisée</v>
       </c>
       <c r="E2" t="str">
-        <v>2026-10-30T23:39:04.193383+00:00</v>
+        <v>2026-10-30T23:47:39.769633+00:00</v>
       </c>
       <c r="F2" t="str">
         <v/>
@@ -563,7 +563,7 @@
         <v>Observation limitée : 1 moto(s), 1 intervalle(s) plein à plein. Ces valeurs décrivent le pilote ; elles ne constituent pas une référence statistique.</v>
       </c>
       <c r="B2" t="str">
-        <v>2026-10-30T23:39:14.990Z</v>
+        <v>2026-10-30T23:47:49.705Z</v>
       </c>
       <c r="C2" t="str">
         <v>BM E2E FICTIF</v>
@@ -617,7 +617,7 @@
         <v>3.5</v>
       </c>
       <c r="F2" t="str">
-        <v>2026-10-30T23:39:02.928+00:00</v>
+        <v>2026-10-30T23:47:38.54+00:00</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
AFLP Moto Manager : photo réelle APSONIC AP150-30 sur la carte du portail
Photo fournie par M. KOUASSI, recadrée 16:9 et compressée en WebP (41 Ko).
Illustration SVG provisoire retirée. Vérifié à 390, 768 et 1440 px.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01YFAq1f7wanW5Hm7vGnu6CV
</commit_message>
<xml_diff>
--- a/tests/moto/resultats/export-pilotage-e2e.xlsx
+++ b/tests/moto/resultats/export-pilotage-e2e.xlsx
@@ -479,7 +479,7 @@
         <v>UH SAKASSOU E2E FICTIF</v>
       </c>
       <c r="K2" t="str">
-        <v>2026-10-30T23:47:33.091473+00:00</v>
+        <v>2026-10-31T00:00:22.210188+00:00</v>
       </c>
       <c r="L2">
         <v>160</v>
@@ -530,7 +530,7 @@
         <v>Immobilisée</v>
       </c>
       <c r="E2" t="str">
-        <v>2026-10-30T23:47:39.769633+00:00</v>
+        <v>2026-10-31T00:00:28.694443+00:00</v>
       </c>
       <c r="F2" t="str">
         <v/>
@@ -563,7 +563,7 @@
         <v>Observation limitée : 1 moto(s), 1 intervalle(s) plein à plein. Ces valeurs décrivent le pilote ; elles ne constituent pas une référence statistique.</v>
       </c>
       <c r="B2" t="str">
-        <v>2026-10-30T23:47:49.705Z</v>
+        <v>2026-10-31T00:00:38.461Z</v>
       </c>
       <c r="C2" t="str">
         <v>BM E2E FICTIF</v>
@@ -617,7 +617,7 @@
         <v>3.5</v>
       </c>
       <c r="F2" t="str">
-        <v>2026-10-30T23:47:38.54+00:00</v>
+        <v>2026-10-31T00:00:27.376+00:00</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
AFLP FLEET : interface, coordination logistique, inspections, corrections de la revue indépendante
- Identité AFLP FLEET (portail, en-tête, exports), routes /moto/ inchangées
- Photo principale avec aperçu, galerie datée, QR vers la fiche
- Acquisition prévue, réception, intégration d'une moto en exploitation sans historique inventé
- État contradictoire avant remise confirmé par le bénéficiaire
- Inspections mensuelles Chef de zone / coordinateur / contrôle indépendant, comparaison
- Actions correctives tracées jusqu'à vérification par un tiers
- Espace Coordination, enveloppes et dépenses, exceptions du Branch Manager
- Revue indépendante : 7 défauts corrigés (indépendance de l'affectataire, photos, justificatifs, stockage)
Recette : serveur 318/318, unitaires 17/17, navigateur 69/69 (0 erreur console), retour arrière vérifié.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01YFAq1f7wanW5Hm7vGnu6CV
</commit_message>
<xml_diff>
--- a/tests/moto/resultats/export-pilotage-e2e.xlsx
+++ b/tests/moto/resultats/export-pilotage-e2e.xlsx
@@ -3,17 +3,18 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <workbookPr codeName="ThisWorkbook"/>
   <sheets>
-    <sheet name="Flotte" sheetId="1" r:id="rId1"/>
-    <sheet name="Consommation" sheetId="2" r:id="rId2"/>
-    <sheet name="Intervalles plein a plein" sheetId="3" r:id="rId3"/>
-    <sheet name="Couts" sheetId="4" r:id="rId4"/>
-    <sheet name="Disponibilite" sheetId="5" r:id="rId5"/>
-    <sheet name="Rapprochement dotations" sheetId="6" r:id="rId6"/>
-    <sheet name="Echeances" sheetId="7" r:id="rId7"/>
-    <sheet name="Alertes documents" sheetId="8" r:id="rId8"/>
-    <sheet name="Pneus" sheetId="9" r:id="rId9"/>
-    <sheet name="Incidents ouverts" sheetId="10" r:id="rId10"/>
-    <sheet name="Limites" sheetId="11" r:id="rId11"/>
+    <sheet name="AFLP FLEET" sheetId="1" r:id="rId1"/>
+    <sheet name="Flotte" sheetId="2" r:id="rId2"/>
+    <sheet name="Consommation" sheetId="3" r:id="rId3"/>
+    <sheet name="Intervalles plein a plein" sheetId="4" r:id="rId4"/>
+    <sheet name="Couts" sheetId="5" r:id="rId5"/>
+    <sheet name="Disponibilite" sheetId="6" r:id="rId6"/>
+    <sheet name="Rapprochement dotations" sheetId="7" r:id="rId7"/>
+    <sheet name="Echeances" sheetId="8" r:id="rId8"/>
+    <sheet name="Alertes documents" sheetId="9" r:id="rId9"/>
+    <sheet name="Pneus" sheetId="10" r:id="rId10"/>
+    <sheet name="Incidents ouverts" sheetId="11" r:id="rId11"/>
+    <sheet name="Limites" sheetId="12" r:id="rId12"/>
   </sheets>
 </workbook>
 </file>
@@ -407,92 +408,59 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:L2"/>
-  <sheetData>
-    <row r="1">
-      <c r="A1" t="str">
-        <v>Code</v>
+  <dimension ref="A1:C2"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="str">
+        <v>Rapport</v>
       </c>
       <c r="B1" t="str">
-        <v>Marque</v>
+        <v>Genere</v>
       </c>
       <c r="C1" t="str">
-        <v>Modele</v>
-      </c>
-      <c r="D1" t="str">
-        <v>Immatriculation</v>
-      </c>
-      <c r="E1" t="str">
-        <v>Chassis</v>
-      </c>
-      <c r="F1" t="str">
-        <v>Cluster</v>
-      </c>
-      <c r="G1" t="str">
-        <v>Administratif</v>
-      </c>
-      <c r="H1" t="str">
-        <v>Affectation</v>
-      </c>
-      <c r="I1" t="str">
-        <v>Technique</v>
-      </c>
-      <c r="J1" t="str">
-        <v>Affectataire</v>
-      </c>
-      <c r="K1" t="str">
-        <v>Mise en service</v>
-      </c>
-      <c r="L1" t="str">
-        <v>Compteur km</v>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="str">
-        <v>MOTO-001</v>
+        <v>Par</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="str">
+        <v>AFLP FLEET · Gestion et suivi du parc de motos AFLP</v>
       </c>
       <c r="B2" t="str">
-        <v>APSONIC</v>
+        <v>2026-10-31T13:09:44.152Z</v>
       </c>
       <c r="C2" t="str">
-        <v>AP150-30</v>
-      </c>
-      <c r="D2" t="str">
-        <v>E2E 0001 FICTIF</v>
-      </c>
-      <c r="E2" t="str">
-        <v>E2E-FICTIF-CH-01</v>
-      </c>
-      <c r="F2" t="str">
-        <v>SAKASSOU</v>
-      </c>
-      <c r="G2" t="str">
-        <v>Conforme</v>
-      </c>
-      <c r="H2" t="str">
-        <v>Remise</v>
-      </c>
-      <c r="I2" t="str">
-        <v>Immobilisée</v>
-      </c>
-      <c r="J2" t="str">
-        <v>UH SAKASSOU E2E FICTIF</v>
-      </c>
-      <c r="K2" t="str">
-        <v>2026-10-31T00:00:22.210188+00:00</v>
-      </c>
-      <c r="L2">
-        <v>160</v>
-      </c>
-    </row>
-  </sheetData>
-  <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:L2"/>
+        <v>BM E2E FICTIF</v>
+      </c>
+    </row>
+  </sheetData>
+  <ignoredErrors>
+    <ignoredError numberStoredAsText="1" sqref="A1:C2"/>
   </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:A2"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="str">
+        <v>Information</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="str">
+        <v>Aucune donnée</v>
+      </c>
+    </row>
+  </sheetData>
+  <ignoredErrors>
+    <ignoredError numberStoredAsText="1" sqref="A1:A2"/>
+  </ignoredErrors>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:F2"/>
   <sheetData>
@@ -530,7 +498,7 @@
         <v>Immobilisée</v>
       </c>
       <c r="E2" t="str">
-        <v>2026-10-31T00:00:28.694443+00:00</v>
+        <v>2026-10-31T13:09:30.062047+00:00</v>
       </c>
       <c r="F2" t="str">
         <v/>
@@ -543,7 +511,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:C2"/>
   <sheetData>
@@ -563,7 +531,7 @@
         <v>Observation limitée : 1 moto(s), 1 intervalle(s) plein à plein. Ces valeurs décrivent le pilote ; elles ne constituent pas une référence statistique.</v>
       </c>
       <c r="B2" t="str">
-        <v>2026-10-31T00:00:38.461Z</v>
+        <v>2026-10-31T13:09:44.154Z</v>
       </c>
       <c r="C2" t="str">
         <v>BM E2E FICTIF</v>
@@ -578,6 +546,99 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:M2"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="str">
+        <v>Code</v>
+      </c>
+      <c r="B1" t="str">
+        <v>Situation</v>
+      </c>
+      <c r="C1" t="str">
+        <v>Marque</v>
+      </c>
+      <c r="D1" t="str">
+        <v>Modele</v>
+      </c>
+      <c r="E1" t="str">
+        <v>Immatriculation</v>
+      </c>
+      <c r="F1" t="str">
+        <v>Chassis</v>
+      </c>
+      <c r="G1" t="str">
+        <v>Cluster</v>
+      </c>
+      <c r="H1" t="str">
+        <v>Administratif</v>
+      </c>
+      <c r="I1" t="str">
+        <v>Affectation</v>
+      </c>
+      <c r="J1" t="str">
+        <v>Technique</v>
+      </c>
+      <c r="K1" t="str">
+        <v>Affectataire</v>
+      </c>
+      <c r="L1" t="str">
+        <v>Mise en service</v>
+      </c>
+      <c r="M1" t="str">
+        <v>Compteur km</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="str">
+        <v>MOTO-001</v>
+      </c>
+      <c r="B2" t="str">
+        <v>Affectée, non opérationnelle</v>
+      </c>
+      <c r="C2" t="str">
+        <v>APSONIC</v>
+      </c>
+      <c r="D2" t="str">
+        <v>AP150-30</v>
+      </c>
+      <c r="E2" t="str">
+        <v>E2E 0001 FICTIF</v>
+      </c>
+      <c r="F2" t="str">
+        <v>E2E-FICTIF-CH-01</v>
+      </c>
+      <c r="G2" t="str">
+        <v>SAKASSOU</v>
+      </c>
+      <c r="H2" t="str">
+        <v>Conforme</v>
+      </c>
+      <c r="I2" t="str">
+        <v>Remise</v>
+      </c>
+      <c r="J2" t="str">
+        <v>Immobilisée</v>
+      </c>
+      <c r="K2" t="str">
+        <v>UH SAKASSOU E2E FICTIF</v>
+      </c>
+      <c r="L2" t="str">
+        <v>2026-10-31T13:09:21.830415+00:00</v>
+      </c>
+      <c r="M2">
+        <v>160</v>
+      </c>
+    </row>
+  </sheetData>
+  <ignoredErrors>
+    <ignoredError numberStoredAsText="1" sqref="A1:M2"/>
+  </ignoredErrors>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:F2"/>
   <sheetData>
     <row r="1">
@@ -617,7 +678,7 @@
         <v>3.5</v>
       </c>
       <c r="F2" t="str">
-        <v>2026-10-31T00:00:27.376+00:00</v>
+        <v>2026-10-31T13:09:28.544+00:00</v>
       </c>
     </row>
   </sheetData>
@@ -627,7 +688,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:G2"/>
   <sheetData>
@@ -684,7 +745,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:H2"/>
   <sheetData>
@@ -747,7 +808,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:D2"/>
   <sheetData>
@@ -786,7 +847,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:N2"/>
   <sheetData>
@@ -885,7 +946,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:A2"/>
   <sheetData>
@@ -906,7 +967,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:D4"/>
   <sheetData>
@@ -971,25 +1032,4 @@
     <ignoredError numberStoredAsText="1" sqref="A1:D4"/>
   </ignoredErrors>
 </worksheet>
-</file>
-
-<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:A2"/>
-  <sheetData>
-    <row r="1">
-      <c r="A1" t="str">
-        <v>Information</v>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="str">
-        <v>Aucune donnée</v>
-      </c>
-    </row>
-  </sheetData>
-  <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:A2"/>
-  </ignoredErrors>
-</worksheet>
 </file>
</xml_diff>

<commit_message>
AFLP FLEET phase 2 : espace Maintenance (tableau du coordinateur, Décisions à prendre du BM, dossiers, garages, règles versionnées)
- Nouveau module moto/moto-maintenance.js, branché sur moto-app.js.
- Droits d'interface alignés sur le serveur : seul le BM autorise une
  dépense ; ZONE et ABM n'ont plus de bouton de décision.
- Circuit incident : plus de montant saisi, constat d'une autorisation BM.
- Recette navigateur 87/87 aux trois largeurs, 0 erreur console.
- Réplique de test alignée sur la production (jit = off).

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01YFAq1f7wanW5Hm7vGnu6CV
</commit_message>
<xml_diff>
--- a/tests/moto/resultats/export-pilotage-e2e.xlsx
+++ b/tests/moto/resultats/export-pilotage-e2e.xlsx
@@ -426,7 +426,7 @@
         <v>AFLP FLEET · Gestion et suivi du parc de motos AFLP</v>
       </c>
       <c r="B2" t="str">
-        <v>2026-10-31T13:09:44.152Z</v>
+        <v>2026-10-31T17:39:32.787Z</v>
       </c>
       <c r="C2" t="str">
         <v>BM E2E FICTIF</v>
@@ -498,7 +498,7 @@
         <v>Immobilisée</v>
       </c>
       <c r="E2" t="str">
-        <v>2026-10-31T13:09:30.062047+00:00</v>
+        <v>2026-10-31T17:39:27.215955+00:00</v>
       </c>
       <c r="F2" t="str">
         <v/>
@@ -531,7 +531,7 @@
         <v>Observation limitée : 1 moto(s), 1 intervalle(s) plein à plein. Ces valeurs décrivent le pilote ; elles ne constituent pas une référence statistique.</v>
       </c>
       <c r="B2" t="str">
-        <v>2026-10-31T13:09:44.154Z</v>
+        <v>2026-10-31T17:39:32.788Z</v>
       </c>
       <c r="C2" t="str">
         <v>BM E2E FICTIF</v>
@@ -624,7 +624,7 @@
         <v>UH SAKASSOU E2E FICTIF</v>
       </c>
       <c r="L2" t="str">
-        <v>2026-10-31T13:09:21.830415+00:00</v>
+        <v>2026-10-31T17:39:19.102466+00:00</v>
       </c>
       <c r="M2">
         <v>160</v>
@@ -678,7 +678,7 @@
         <v>3.5</v>
       </c>
       <c r="F2" t="str">
-        <v>2026-10-31T13:09:28.544+00:00</v>
+        <v>2026-10-31T17:39:25.707+00:00</v>
       </c>
     </row>
   </sheetData>
@@ -948,21 +948,64 @@
 
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:A2"/>
-  <sheetData>
-    <row r="1">
-      <c r="A1" t="str">
-        <v>Information</v>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="str">
-        <v>Aucune donnée</v>
-      </c>
-    </row>
-  </sheetData>
-  <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:A2"/>
+  <dimension ref="A1:F4"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="str">
+        <v>Moto</v>
+      </c>
+      <c r="B1" t="str">
+        <v>Regle</v>
+      </c>
+      <c r="C1" t="str">
+        <v>Source</v>
+      </c>
+      <c r="D1" t="str">
+        <v>Prochaine km</v>
+      </c>
+      <c r="E1" t="str">
+        <v>Prochaine date</v>
+      </c>
+      <c r="F1" t="str">
+        <v>Statut</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="str">
+        <v>MOTO-001</v>
+      </c>
+      <c r="B2" t="str">
+        <v>Vidange huile moteur</v>
+      </c>
+      <c r="F2" t="str">
+        <v>DIAGNOSTIC_INITIAL_REQUIS</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="str">
+        <v>MOTO-001</v>
+      </c>
+      <c r="B3" t="str">
+        <v>Entretien préventif (chaîne, freins, filtres)</v>
+      </c>
+      <c r="F3" t="str">
+        <v>DIAGNOSTIC_INITIAL_REQUIS</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="str">
+        <v>MOTO-001</v>
+      </c>
+      <c r="B4" t="str">
+        <v>Révision générale</v>
+      </c>
+      <c r="F4" t="str">
+        <v>DIAGNOSTIC_INITIAL_REQUIS</v>
+      </c>
+    </row>
+  </sheetData>
+  <ignoredErrors>
+    <ignoredError numberStoredAsText="1" sqref="A1:F4"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
AFLP FLEET phase 2 : verrous contre le double règlement et la double vérification concurrents
- Facture verrouillée avant tout calcul de reste dû (paiement Finance,
  règlement par enveloppe, répartition de pneus).
- Dossier verrouillé avant le cumul des factures vérifiées ; une facture
  n'est couverte que par les autorisations décidées au plus tard à sa date.
- Aucun engagement chez un garage suspendu après la décision.
- Tests de concurrence réels (deux sessions simultanées) : échouent sans les
  verrous (preuve : resultats/maintenance_6_preuve_sans_verrous.json,
  10 000 réglés et 10 000 vérifiés pour 5 000), passent avec.
- Recette : 352/352, 202/202, 87/87, retour arrière prouvé.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01YFAq1f7wanW5Hm7vGnu6CV
</commit_message>
<xml_diff>
--- a/tests/moto/resultats/export-pilotage-e2e.xlsx
+++ b/tests/moto/resultats/export-pilotage-e2e.xlsx
@@ -426,7 +426,7 @@
         <v>AFLP FLEET · Gestion et suivi du parc de motos AFLP</v>
       </c>
       <c r="B2" t="str">
-        <v>2026-10-31T18:07:41.958Z</v>
+        <v>2026-10-31T18:24:41.311Z</v>
       </c>
       <c r="C2" t="str">
         <v>BM E2E FICTIF</v>
@@ -498,7 +498,7 @@
         <v>Immobilisée</v>
       </c>
       <c r="E2" t="str">
-        <v>2026-10-31T18:07:36.599104+00:00</v>
+        <v>2026-10-31T18:24:36.417252+00:00</v>
       </c>
       <c r="F2" t="str">
         <v/>
@@ -531,7 +531,7 @@
         <v>Observation limitée : 1 moto(s), 1 intervalle(s) plein à plein. Ces valeurs décrivent le pilote ; elles ne constituent pas une référence statistique.</v>
       </c>
       <c r="B2" t="str">
-        <v>2026-10-31T18:07:41.961Z</v>
+        <v>2026-10-31T18:24:41.313Z</v>
       </c>
       <c r="C2" t="str">
         <v>BM E2E FICTIF</v>
@@ -624,7 +624,7 @@
         <v>UH SAKASSOU E2E FICTIF</v>
       </c>
       <c r="L2" t="str">
-        <v>2026-10-31T18:07:28.711656+00:00</v>
+        <v>2026-10-31T18:24:28.369515+00:00</v>
       </c>
       <c r="M2">
         <v>160</v>
@@ -678,7 +678,7 @@
         <v>3.5</v>
       </c>
       <c r="F2" t="str">
-        <v>2026-10-31T18:07:35.039+00:00</v>
+        <v>2026-10-31T18:24:34.931+00:00</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
AFLP FLEET phase 2 : libellés de réparation refusés en supervision (décision BM), ordre de verrouillage unique, rapport de contre-expertise
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01YFAq1f7wanW5Hm7vGnu6CV
</commit_message>
<xml_diff>
--- a/tests/moto/resultats/export-pilotage-e2e.xlsx
+++ b/tests/moto/resultats/export-pilotage-e2e.xlsx
@@ -426,7 +426,7 @@
         <v>AFLP FLEET · Gestion et suivi du parc de motos AFLP</v>
       </c>
       <c r="B2" t="str">
-        <v>2026-10-31T18:24:41.311Z</v>
+        <v>2026-10-31T18:40:47.307Z</v>
       </c>
       <c r="C2" t="str">
         <v>BM E2E FICTIF</v>
@@ -498,7 +498,7 @@
         <v>Immobilisée</v>
       </c>
       <c r="E2" t="str">
-        <v>2026-10-31T18:24:36.417252+00:00</v>
+        <v>2026-10-31T18:40:42.332708+00:00</v>
       </c>
       <c r="F2" t="str">
         <v/>
@@ -531,7 +531,7 @@
         <v>Observation limitée : 1 moto(s), 1 intervalle(s) plein à plein. Ces valeurs décrivent le pilote ; elles ne constituent pas une référence statistique.</v>
       </c>
       <c r="B2" t="str">
-        <v>2026-10-31T18:24:41.313Z</v>
+        <v>2026-10-31T18:40:47.309Z</v>
       </c>
       <c r="C2" t="str">
         <v>BM E2E FICTIF</v>
@@ -624,7 +624,7 @@
         <v>UH SAKASSOU E2E FICTIF</v>
       </c>
       <c r="L2" t="str">
-        <v>2026-10-31T18:24:28.369515+00:00</v>
+        <v>2026-10-31T18:40:34.720952+00:00</v>
       </c>
       <c r="M2">
         <v>160</v>
@@ -678,7 +678,7 @@
         <v>3.5</v>
       </c>
       <c r="F2" t="str">
-        <v>2026-10-31T18:24:34.931+00:00</v>
+        <v>2026-10-31T18:40:40.915+00:00</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
AFLP FLEET : export de pilotage régénéré par la recette navigateur sur main (87/87)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01YFAq1gjG8bCE79e74sYNuh
</commit_message>
<xml_diff>
--- a/tests/moto/resultats/export-pilotage-e2e.xlsx
+++ b/tests/moto/resultats/export-pilotage-e2e.xlsx
@@ -426,7 +426,7 @@
         <v>AFLP FLEET · Gestion et suivi du parc de motos AFLP</v>
       </c>
       <c r="B2" t="str">
-        <v>2026-10-31T18:40:47.307Z</v>
+        <v>2026-10-31T20:20:42.405Z</v>
       </c>
       <c r="C2" t="str">
         <v>BM E2E FICTIF</v>
@@ -498,7 +498,7 @@
         <v>Immobilisée</v>
       </c>
       <c r="E2" t="str">
-        <v>2026-10-31T18:40:42.332708+00:00</v>
+        <v>2026-10-31T20:20:38.977773+00:00</v>
       </c>
       <c r="F2" t="str">
         <v/>
@@ -531,7 +531,7 @@
         <v>Observation limitée : 1 moto(s), 1 intervalle(s) plein à plein. Ces valeurs décrivent le pilote ; elles ne constituent pas une référence statistique.</v>
       </c>
       <c r="B2" t="str">
-        <v>2026-10-31T18:40:47.309Z</v>
+        <v>2026-10-31T20:20:42.406Z</v>
       </c>
       <c r="C2" t="str">
         <v>BM E2E FICTIF</v>
@@ -624,7 +624,7 @@
         <v>UH SAKASSOU E2E FICTIF</v>
       </c>
       <c r="L2" t="str">
-        <v>2026-10-31T18:40:34.720952+00:00</v>
+        <v>2026-10-31T20:20:33.564843+00:00</v>
       </c>
       <c r="M2">
         <v>160</v>
@@ -678,7 +678,7 @@
         <v>3.5</v>
       </c>
       <c r="F2" t="str">
-        <v>2026-10-31T18:40:40.915+00:00</v>
+        <v>2026-10-31T20:20:37.872+00:00</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
AFLP FLEET migration 7 : un permis retiré ne se réactive pas par redépôt (contre-vérification)
- Numéro retiré bloqué au dépôt et à la vérification, quel que soit le
  titulaire ; levée réservée au BM (motif), sans rendre le permis valide.
- Historique de retrait visible dans la vue et la fenêtre de vérification.
- Garde de remise limitée aux affectations actives (purge possible) ; relecture
  du permis valide après verrou (renouvellement simultané).
Recette : 352/352, 204/204, 115/115, navigateur 102/102, retour arrière prouvé.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01YFAq1gjG8bCE79e74sYNuh
</commit_message>
<xml_diff>
--- a/tests/moto/resultats/export-pilotage-e2e.xlsx
+++ b/tests/moto/resultats/export-pilotage-e2e.xlsx
@@ -426,7 +426,7 @@
         <v>AFLP FLEET · Gestion et suivi du parc de motos AFLP</v>
       </c>
       <c r="B2" t="str">
-        <v>2026-11-01T08:37:04.506Z</v>
+        <v>2026-11-01T08:43:47.991Z</v>
       </c>
       <c r="C2" t="str">
         <v>BM E2E FICTIF</v>
@@ -498,7 +498,7 @@
         <v>Immobilisée</v>
       </c>
       <c r="E2" t="str">
-        <v>2026-11-01T08:37:00.873103+00:00</v>
+        <v>2026-11-01T08:43:44.421301+00:00</v>
       </c>
       <c r="F2" t="str">
         <v/>
@@ -531,7 +531,7 @@
         <v>Observation limitée : 1 moto(s), 1 intervalle(s) plein à plein. Ces valeurs décrivent le pilote ; elles ne constituent pas une référence statistique.</v>
       </c>
       <c r="B2" t="str">
-        <v>2026-11-01T08:37:04.507Z</v>
+        <v>2026-11-01T08:43:47.992Z</v>
       </c>
       <c r="C2" t="str">
         <v>BM E2E FICTIF</v>
@@ -624,7 +624,7 @@
         <v>UH SAKASSOU E2E FICTIF</v>
       </c>
       <c r="L2" t="str">
-        <v>2026-11-01T08:36:55.270359+00:00</v>
+        <v>2026-11-01T08:43:38.852826+00:00</v>
       </c>
       <c r="M2">
         <v>160</v>
@@ -678,7 +678,7 @@
         <v>3.5</v>
       </c>
       <c r="F2" t="str">
-        <v>2026-11-01T08:36:59.71+00:00</v>
+        <v>2026-11-01T08:43:43.277+00:00</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
AFLP FLEET migration 7 : numéro réservé à son titulaire, quatre yeux après levée, ordre des verrous
- Un numéro de permis appartient à une seule personne : réservé dès son dépôt
  (hors dépôt rejeté), même retiré, levé ou remplacé.
- Quatre yeux : qui a levé un retrait ne vérifie pas le redépôt (l'ABM le fait).
- Ordre de verrouillage commun (numéro, puis ligne) dans vérifier, retirer,
  lever : aucun interblocage entre retrait et vérification simultanés (prouvé).
Recette : 352/352, 204/204, 118/118, navigateur 102/102, retour arrière prouvé.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01YFAq1gjG8bCE79e74sYNuh
</commit_message>
<xml_diff>
--- a/tests/moto/resultats/export-pilotage-e2e.xlsx
+++ b/tests/moto/resultats/export-pilotage-e2e.xlsx
@@ -426,7 +426,7 @@
         <v>AFLP FLEET · Gestion et suivi du parc de motos AFLP</v>
       </c>
       <c r="B2" t="str">
-        <v>2026-11-01T08:43:47.991Z</v>
+        <v>2026-11-01T08:51:16.668Z</v>
       </c>
       <c r="C2" t="str">
         <v>BM E2E FICTIF</v>
@@ -498,7 +498,7 @@
         <v>Immobilisée</v>
       </c>
       <c r="E2" t="str">
-        <v>2026-11-01T08:43:44.421301+00:00</v>
+        <v>2026-11-01T08:51:13.086897+00:00</v>
       </c>
       <c r="F2" t="str">
         <v/>
@@ -531,7 +531,7 @@
         <v>Observation limitée : 1 moto(s), 1 intervalle(s) plein à plein. Ces valeurs décrivent le pilote ; elles ne constituent pas une référence statistique.</v>
       </c>
       <c r="B2" t="str">
-        <v>2026-11-01T08:43:47.992Z</v>
+        <v>2026-11-01T08:51:16.669Z</v>
       </c>
       <c r="C2" t="str">
         <v>BM E2E FICTIF</v>
@@ -624,7 +624,7 @@
         <v>UH SAKASSOU E2E FICTIF</v>
       </c>
       <c r="L2" t="str">
-        <v>2026-11-01T08:43:38.852826+00:00</v>
+        <v>2026-11-01T08:51:07.274696+00:00</v>
       </c>
       <c r="M2">
         <v>160</v>
@@ -678,7 +678,7 @@
         <v>3.5</v>
       </c>
       <c r="F2" t="str">
-        <v>2026-11-01T08:43:43.277+00:00</v>
+        <v>2026-11-01T08:51:11.876+00:00</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
AFLP FLEET migration 7 : annulation d'un permis validé pour une mauvaise personne
moto_permis_annuler_erreur : Branch Manager seul, motif détaillé, quatre yeux
(ni le vérificateur ni le titulaire) ; statut ANNULE, numéro libéré pour le
vrai titulaire. Recette : 352/352, 204/204, 129/129, navigateur 102/102,
retour arrière prouvé.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01YFAq1gjG8bCE79e74sYNuh
</commit_message>
<xml_diff>
--- a/tests/moto/resultats/export-pilotage-e2e.xlsx
+++ b/tests/moto/resultats/export-pilotage-e2e.xlsx
@@ -426,7 +426,7 @@
         <v>AFLP FLEET · Gestion et suivi du parc de motos AFLP</v>
       </c>
       <c r="B2" t="str">
-        <v>2026-11-01T08:51:16.668Z</v>
+        <v>2026-11-01T08:56:22.873Z</v>
       </c>
       <c r="C2" t="str">
         <v>BM E2E FICTIF</v>
@@ -498,7 +498,7 @@
         <v>Immobilisée</v>
       </c>
       <c r="E2" t="str">
-        <v>2026-11-01T08:51:13.086897+00:00</v>
+        <v>2026-11-01T08:56:19.136228+00:00</v>
       </c>
       <c r="F2" t="str">
         <v/>
@@ -531,7 +531,7 @@
         <v>Observation limitée : 1 moto(s), 1 intervalle(s) plein à plein. Ces valeurs décrivent le pilote ; elles ne constituent pas une référence statistique.</v>
       </c>
       <c r="B2" t="str">
-        <v>2026-11-01T08:51:16.669Z</v>
+        <v>2026-11-01T08:56:22.874Z</v>
       </c>
       <c r="C2" t="str">
         <v>BM E2E FICTIF</v>
@@ -624,7 +624,7 @@
         <v>UH SAKASSOU E2E FICTIF</v>
       </c>
       <c r="L2" t="str">
-        <v>2026-11-01T08:51:07.274696+00:00</v>
+        <v>2026-11-01T08:56:13.541053+00:00</v>
       </c>
       <c r="M2">
         <v>160</v>
@@ -678,7 +678,7 @@
         <v>3.5</v>
       </c>
       <c r="F2" t="str">
-        <v>2026-11-01T08:51:11.876+00:00</v>
+        <v>2026-11-01T08:56:17.963+00:00</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
AFLP FLEET migration 7 : qui annule un permis ne valide pas le dépôt suivant sur ce numéro
Quatre yeux sur le numéro : un Branch Manager seul ne peut plus faire passer
le numéro d'un vrai titulaire à un tiers (annulation puis validation).
Motif de l'annulation tracé au journal (test W13).
Recette : 352/352, 204/204, 132/132, navigateur 102/102, retour arrière prouvé.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01YFAq1gjG8bCE79e74sYNuh
</commit_message>
<xml_diff>
--- a/tests/moto/resultats/export-pilotage-e2e.xlsx
+++ b/tests/moto/resultats/export-pilotage-e2e.xlsx
@@ -426,7 +426,7 @@
         <v>AFLP FLEET · Gestion et suivi du parc de motos AFLP</v>
       </c>
       <c r="B2" t="str">
-        <v>2026-11-01T08:56:22.873Z</v>
+        <v>2026-11-01T09:00:46.445Z</v>
       </c>
       <c r="C2" t="str">
         <v>BM E2E FICTIF</v>
@@ -498,7 +498,7 @@
         <v>Immobilisée</v>
       </c>
       <c r="E2" t="str">
-        <v>2026-11-01T08:56:19.136228+00:00</v>
+        <v>2026-11-01T09:00:43.106069+00:00</v>
       </c>
       <c r="F2" t="str">
         <v/>
@@ -531,7 +531,7 @@
         <v>Observation limitée : 1 moto(s), 1 intervalle(s) plein à plein. Ces valeurs décrivent le pilote ; elles ne constituent pas une référence statistique.</v>
       </c>
       <c r="B2" t="str">
-        <v>2026-11-01T08:56:22.874Z</v>
+        <v>2026-11-01T09:00:46.446Z</v>
       </c>
       <c r="C2" t="str">
         <v>BM E2E FICTIF</v>
@@ -624,7 +624,7 @@
         <v>UH SAKASSOU E2E FICTIF</v>
       </c>
       <c r="L2" t="str">
-        <v>2026-11-01T08:56:13.541053+00:00</v>
+        <v>2026-11-01T09:00:37.417307+00:00</v>
       </c>
       <c r="M2">
         <v>160</v>
@@ -678,7 +678,7 @@
         <v>3.5</v>
       </c>
       <c r="F2" t="str">
-        <v>2026-11-01T08:56:17.963+00:00</v>
+        <v>2026-11-01T09:00:41.92+00:00</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
AFLP FLEET migration 7 : qui a libéré un numéro ne le réattribue pas seul
Quatre yeux généralisé : la personne qui a libéré un numéro (annulation, ou
rejet du dépôt d'une autre personne) ne valide pas un dépôt portant ce numéro ;
un numéro disputé entre deux personnes est tranché par l'ABM.
Recette : 352/352, 204/204, 140/140, navigateur 102/102, retour arrière prouvé.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01YFAq1gjG8bCE79e74sYNuh
</commit_message>
<xml_diff>
--- a/tests/moto/resultats/export-pilotage-e2e.xlsx
+++ b/tests/moto/resultats/export-pilotage-e2e.xlsx
@@ -426,7 +426,7 @@
         <v>AFLP FLEET · Gestion et suivi du parc de motos AFLP</v>
       </c>
       <c r="B2" t="str">
-        <v>2026-11-01T09:00:46.445Z</v>
+        <v>2026-11-01T09:05:57.430Z</v>
       </c>
       <c r="C2" t="str">
         <v>BM E2E FICTIF</v>
@@ -498,7 +498,7 @@
         <v>Immobilisée</v>
       </c>
       <c r="E2" t="str">
-        <v>2026-11-01T09:00:43.106069+00:00</v>
+        <v>2026-11-01T09:05:53.441855+00:00</v>
       </c>
       <c r="F2" t="str">
         <v/>
@@ -531,7 +531,7 @@
         <v>Observation limitée : 1 moto(s), 1 intervalle(s) plein à plein. Ces valeurs décrivent le pilote ; elles ne constituent pas une référence statistique.</v>
       </c>
       <c r="B2" t="str">
-        <v>2026-11-01T09:00:46.446Z</v>
+        <v>2026-11-01T09:05:57.432Z</v>
       </c>
       <c r="C2" t="str">
         <v>BM E2E FICTIF</v>
@@ -624,7 +624,7 @@
         <v>UH SAKASSOU E2E FICTIF</v>
       </c>
       <c r="L2" t="str">
-        <v>2026-11-01T09:00:37.417307+00:00</v>
+        <v>2026-11-01T09:05:47.534856+00:00</v>
       </c>
       <c r="M2">
         <v>160</v>
@@ -678,7 +678,7 @@
         <v>3.5</v>
       </c>
       <c r="F2" t="str">
-        <v>2026-11-01T09:00:41.92+00:00</v>
+        <v>2026-11-01T09:05:52.274+00:00</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
AFLP FLEET migration 8 : journal de mission et kilométrage contrôlé par photo
- Missions départ/arrivée : compteur + photo du compteur (caméra FIELD PROOF), empreinte unique,
  positions GPS séparées (jamais lisibles par la Finance ni la Direction, jamais journalisées)
- Lecture gratuite du compteur sur le téléphone : la machine propose, l'agent confirme
- Écarts à vérifier (hors mission, continuité, vitesse, distance, horloge, GPS, clôture tardive)
- Tableaux de bord, coût par km de mission, export Excel ; carnet de suivi enrichi
- Tests : 352 + 204 + 140 + 112 serveur, 117/117 navigateur, retour arrière prouvé
- Contre-expertise indépendante en cours ; migration NON appliquée en production

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01YFAq1gjG8bCE79e74sYNuh
</commit_message>
<xml_diff>
--- a/tests/moto/resultats/export-pilotage-e2e.xlsx
+++ b/tests/moto/resultats/export-pilotage-e2e.xlsx
@@ -426,7 +426,7 @@
         <v>AFLP FLEET · Gestion et suivi du parc de motos AFLP</v>
       </c>
       <c r="B2" t="str">
-        <v>2026-11-01T09:05:57.430Z</v>
+        <v>2026-11-01T12:28:07.309Z</v>
       </c>
       <c r="C2" t="str">
         <v>BM E2E FICTIF</v>
@@ -498,7 +498,7 @@
         <v>Immobilisée</v>
       </c>
       <c r="E2" t="str">
-        <v>2026-11-01T09:05:53.441855+00:00</v>
+        <v>2026-11-01T12:28:04.033963+00:00</v>
       </c>
       <c r="F2" t="str">
         <v/>
@@ -531,7 +531,7 @@
         <v>Observation limitée : 1 moto(s), 1 intervalle(s) plein à plein. Ces valeurs décrivent le pilote ; elles ne constituent pas une référence statistique.</v>
       </c>
       <c r="B2" t="str">
-        <v>2026-11-01T09:05:57.432Z</v>
+        <v>2026-11-01T12:28:07.310Z</v>
       </c>
       <c r="C2" t="str">
         <v>BM E2E FICTIF</v>
@@ -624,7 +624,7 @@
         <v>UH SAKASSOU E2E FICTIF</v>
       </c>
       <c r="L2" t="str">
-        <v>2026-11-01T09:05:47.534856+00:00</v>
+        <v>2026-11-01T12:27:58.772382+00:00</v>
       </c>
       <c r="M2">
         <v>160</v>
@@ -678,7 +678,7 @@
         <v>3.5</v>
       </c>
       <c r="F2" t="str">
-        <v>2026-11-01T09:05:52.274+00:00</v>
+        <v>2026-11-01T12:28:03.035+00:00</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
AFLP FLEET migration 8 : corrections de la contre-expertise (3 bloquants, 6 majeurs, mineurs)
- Compteur NaN/infini refusé (moto_num) ; départ antidaté, chevauchement et permis expiré refusés
- Réutilisation d'un même fichier détectée par l'eTag du stockage ; écart SAISIE_DIFFEREE
- Arrivée reçue avant son départ : erreur temporaire, jamais rejet définitif (serveur et file locale)
- Km hors mission non doublés après annulation ; continuité contrôlée à chaque correction
- Chef de zone limité à sa zone pour missions, positions, annulation et écarts
- Verrou moto d'abord dans moto_correction_decider ; conducteur exclu de la validation
- Photos de mission lisibles seulement par qui lit la mission ; purge BM ; retour arrière rejouable
- Tests : 352 + 204 + 140 + 143 serveur, 117/117 navigateur, retour arrière prouvé

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01YFAq1gjG8bCE79e74sYNuh
</commit_message>
<xml_diff>
--- a/tests/moto/resultats/export-pilotage-e2e.xlsx
+++ b/tests/moto/resultats/export-pilotage-e2e.xlsx
@@ -426,7 +426,7 @@
         <v>AFLP FLEET · Gestion et suivi du parc de motos AFLP</v>
       </c>
       <c r="B2" t="str">
-        <v>2026-11-01T12:28:07.309Z</v>
+        <v>2026-11-01T12:48:52.331Z</v>
       </c>
       <c r="C2" t="str">
         <v>BM E2E FICTIF</v>
@@ -498,7 +498,7 @@
         <v>Immobilisée</v>
       </c>
       <c r="E2" t="str">
-        <v>2026-11-01T12:28:04.033963+00:00</v>
+        <v>2026-11-01T12:48:49.03889+00:00</v>
       </c>
       <c r="F2" t="str">
         <v/>
@@ -531,7 +531,7 @@
         <v>Observation limitée : 1 moto(s), 1 intervalle(s) plein à plein. Ces valeurs décrivent le pilote ; elles ne constituent pas une référence statistique.</v>
       </c>
       <c r="B2" t="str">
-        <v>2026-11-01T12:28:07.310Z</v>
+        <v>2026-11-01T12:48:52.333Z</v>
       </c>
       <c r="C2" t="str">
         <v>BM E2E FICTIF</v>
@@ -624,7 +624,7 @@
         <v>UH SAKASSOU E2E FICTIF</v>
       </c>
       <c r="L2" t="str">
-        <v>2026-11-01T12:27:58.772382+00:00</v>
+        <v>2026-11-01T12:48:43.971196+00:00</v>
       </c>
       <c r="M2">
         <v>160</v>
@@ -678,7 +678,7 @@
         <v>3.5</v>
       </c>
       <c r="F2" t="str">
-        <v>2026-11-01T12:28:03.035+00:00</v>
+        <v>2026-11-01T12:48:47.969+00:00</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
AFLP FLEET migration 8 : corrections de la contre-vérification (régressions R1 à R5)
- Saisies hors connexion reçues dans le désordre : acceptées et signalées (ORDRE_RELEVES), seul le chevauchement est refusé
- Tolérance d'horloge 15 min (écart HORLOGE signalé) ; eTag du stockage obligatoire
- Purge : plancher de 12 mois codé en dur, quel que soit le paramètre
- Contrôle d'empreinte par un tiers (moto_mission_photo_controler, écart EMPREINTE_DIFFERENTE) ; photos atypiques signalées
- Carnet : missions filtrées comme leur lecture ; arrivée orpheline marquée refusée sur l'appareil
- Tests : 352 + 204 + 140 + 160 serveur, 117/117 navigateur, retour arrière prouvé

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01YFAq1gjG8bCE79e74sYNuh
</commit_message>
<xml_diff>
--- a/tests/moto/resultats/export-pilotage-e2e.xlsx
+++ b/tests/moto/resultats/export-pilotage-e2e.xlsx
@@ -426,7 +426,7 @@
         <v>AFLP FLEET · Gestion et suivi du parc de motos AFLP</v>
       </c>
       <c r="B2" t="str">
-        <v>2026-11-01T12:48:52.331Z</v>
+        <v>2026-11-01T12:59:52.946Z</v>
       </c>
       <c r="C2" t="str">
         <v>BM E2E FICTIF</v>
@@ -498,7 +498,7 @@
         <v>Immobilisée</v>
       </c>
       <c r="E2" t="str">
-        <v>2026-11-01T12:48:49.03889+00:00</v>
+        <v>2026-11-01T12:59:49.671234+00:00</v>
       </c>
       <c r="F2" t="str">
         <v/>
@@ -531,7 +531,7 @@
         <v>Observation limitée : 1 moto(s), 1 intervalle(s) plein à plein. Ces valeurs décrivent le pilote ; elles ne constituent pas une référence statistique.</v>
       </c>
       <c r="B2" t="str">
-        <v>2026-11-01T12:48:52.333Z</v>
+        <v>2026-11-01T12:59:52.948Z</v>
       </c>
       <c r="C2" t="str">
         <v>BM E2E FICTIF</v>
@@ -624,7 +624,7 @@
         <v>UH SAKASSOU E2E FICTIF</v>
       </c>
       <c r="L2" t="str">
-        <v>2026-11-01T12:48:43.971196+00:00</v>
+        <v>2026-11-01T12:59:44.576972+00:00</v>
       </c>
       <c r="M2">
         <v>160</v>
@@ -678,7 +678,7 @@
         <v>3.5</v>
       </c>
       <c r="F2" t="str">
-        <v>2026-11-01T12:48:47.969+00:00</v>
+        <v>2026-11-01T12:59:48.61+00:00</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
AFLP FLEET migration 8 : réserve N1 levée (chevauchement par intervalle) et levée motivée d'un contrôle infondé
- Départ refusé seulement s'il tombe PENDANT une mission ; mission plus ancienne saisie hors connexion acceptée
  (erreur temporaire si une mission plus récente est encore ouverte) ; arrivée refusée si une autre mission part entre-temps
- Heure de capture en avance ramenée à l'heure du serveur (écart HORLOGE conservé)
- Historique des contrôles d'empreinte ; levée d'un non-conforme par BM/ABM, quatre yeux, motif
- Tests : 352 + 204 + 140 + 175 serveur, 117/117 navigateur, retour arrière prouvé

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01YFAq1gjG8bCE79e74sYNuh
</commit_message>
<xml_diff>
--- a/tests/moto/resultats/export-pilotage-e2e.xlsx
+++ b/tests/moto/resultats/export-pilotage-e2e.xlsx
@@ -426,7 +426,7 @@
         <v>AFLP FLEET · Gestion et suivi du parc de motos AFLP</v>
       </c>
       <c r="B2" t="str">
-        <v>2026-11-01T12:59:52.946Z</v>
+        <v>2026-11-01T13:10:23.730Z</v>
       </c>
       <c r="C2" t="str">
         <v>BM E2E FICTIF</v>
@@ -498,7 +498,7 @@
         <v>Immobilisée</v>
       </c>
       <c r="E2" t="str">
-        <v>2026-11-01T12:59:49.671234+00:00</v>
+        <v>2026-11-01T13:10:20.590404+00:00</v>
       </c>
       <c r="F2" t="str">
         <v/>
@@ -531,7 +531,7 @@
         <v>Observation limitée : 1 moto(s), 1 intervalle(s) plein à plein. Ces valeurs décrivent le pilote ; elles ne constituent pas une référence statistique.</v>
       </c>
       <c r="B2" t="str">
-        <v>2026-11-01T12:59:52.948Z</v>
+        <v>2026-11-01T13:10:23.731Z</v>
       </c>
       <c r="C2" t="str">
         <v>BM E2E FICTIF</v>
@@ -624,7 +624,7 @@
         <v>UH SAKASSOU E2E FICTIF</v>
       </c>
       <c r="L2" t="str">
-        <v>2026-11-01T12:59:44.576972+00:00</v>
+        <v>2026-11-01T13:10:15.5222+00:00</v>
       </c>
       <c r="M2">
         <v>160</v>
@@ -678,7 +678,7 @@
         <v>3.5</v>
       </c>
       <c r="F2" t="str">
-        <v>2026-11-01T12:59:48.61+00:00</v>
+        <v>2026-11-01T13:10:19.585+00:00</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
AFLP FLEET migration 8 : arrivée qui chevauche annulée automatiquement (moto jamais bloquée), quatre yeux sur la levée
- Contre-expertise : 4e passage GO ; défaut majeur restant corrigé et testé
- Tests : 352 + 204 + 140 + 180 serveur, 117/117 navigateur, retour arrière prouvé

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01YFAq1gjG8bCE79e74sYNuh
</commit_message>
<xml_diff>
--- a/tests/moto/resultats/export-pilotage-e2e.xlsx
+++ b/tests/moto/resultats/export-pilotage-e2e.xlsx
@@ -426,7 +426,7 @@
         <v>AFLP FLEET · Gestion et suivi du parc de motos AFLP</v>
       </c>
       <c r="B2" t="str">
-        <v>2026-11-01T13:10:23.730Z</v>
+        <v>2026-11-01T13:16:17.711Z</v>
       </c>
       <c r="C2" t="str">
         <v>BM E2E FICTIF</v>
@@ -498,7 +498,7 @@
         <v>Immobilisée</v>
       </c>
       <c r="E2" t="str">
-        <v>2026-11-01T13:10:20.590404+00:00</v>
+        <v>2026-11-01T13:16:14.530664+00:00</v>
       </c>
       <c r="F2" t="str">
         <v/>
@@ -531,7 +531,7 @@
         <v>Observation limitée : 1 moto(s), 1 intervalle(s) plein à plein. Ces valeurs décrivent le pilote ; elles ne constituent pas une référence statistique.</v>
       </c>
       <c r="B2" t="str">
-        <v>2026-11-01T13:10:23.731Z</v>
+        <v>2026-11-01T13:16:17.712Z</v>
       </c>
       <c r="C2" t="str">
         <v>BM E2E FICTIF</v>
@@ -624,7 +624,7 @@
         <v>UH SAKASSOU E2E FICTIF</v>
       </c>
       <c r="L2" t="str">
-        <v>2026-11-01T13:10:15.5222+00:00</v>
+        <v>2026-11-01T13:16:09.533165+00:00</v>
       </c>
       <c r="M2">
         <v>160</v>
@@ -678,7 +678,7 @@
         <v>3.5</v>
       </c>
       <c r="F2" t="str">
-        <v>2026-11-01T13:10:19.585+00:00</v>
+        <v>2026-11-01T13:16:13.537+00:00</v>
       </c>
     </row>
   </sheetData>

</xml_diff>